<commit_message>
update base de donnees
</commit_message>
<xml_diff>
--- a/quartier_app/data/precision_overrides.xlsx
+++ b/quartier_app/data/precision_overrides.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,11 +446,7 @@
           <t>1-092||SOPIE||294||VIDE</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paris village</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -459,6 +455,1094 @@
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A276||||241||VIDE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>les versants</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1-115||ORANGE GIB||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Scierie GIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1-115||ORANGE GIB||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Scierie GIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1-374||CITE LES HAUT PLATEAUX DE BINGERVILLE||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CITE LES HAUT PLATEAUX DE BINGERVILLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1-350||JAAFAR||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JAAFAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1-331||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ANAN-CITE PETROCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1-330||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PROGRAMME MOKE G2I</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1-273||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Laurier 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1-306||LAURIER 21||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Laurier 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1-072||SEBIA YAO||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Eglise Évangélique des Élus de Dieu de SEBIA-YAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1-225||LAURIERS 22||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LAURIERS 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1-023 B||ANA VILLAGE||326||VIDE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Église Catholique St Mathieu, Anan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1-167||MARIE LEVY||326||École secondaire</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>École secondaire MARIE LEVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1-078||||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HydroFish</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1-028 B||DJOLO 2||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DJOLO 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1-321||||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Quartier Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1-287||BERLIN||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Quartier BERLIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1-335||EDEN BEACH||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>EDEN BEACH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1-322||||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Quartier Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1-311||ST CYRILE||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Saint Cyrille</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1-127 B||GBAGBA CARIERE||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>GBAGBA CARRIERE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1-071 B||MARCHER BERLIN||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Marché Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1-062 B||EPP MARCHOUX||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MARCHOUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1-042 B||VILLAGE MARCHOUX||325||VIDE</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>VILLAGE MARCHOUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1-219||DJOLO||323||VIDE</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DJOLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1-213||LAURIERS 20||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LAURIERS 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ATELIER CME||ATELIER CME||296||VIDE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ATELIER CME</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ADM CME||CME GUERRITE||311||VIDE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ADM CME</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1-165 B||GBAGBA EXTENTION||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>GBAGBA EXTENTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1-049 B||CAMILLE ALIALI||327||VIDE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SABLIERE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1-249||||322||VIDE</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LAURIER 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R56||M'POUTO||287||Maquis La Cave</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>R56||M'POUTO||287||Centre de santé municipal de M'pouto</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Centre de santé municipal de M'pouto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>R56||M'POUTO||287||Garbadrôme M’Pouto</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1-049 B||CAMILLA ALIALI||327||VIDE</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Cité KELATY-Sablière</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1-310||||312||VIDE</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Harris</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1-343||GBAGBA||325||VIDE</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Machoux</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1-050||SICOGI 1||316||VIDE</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SICOGI 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1-444||||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Abatta BCEAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>R471||FAYA HOPITAL||243||Pressing Gymek</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Ephrata</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>R471||FAYA HOPITAL||243||Cave la Terrasse</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>R471||FAYA HOPITAL||243||Maquis Les délice du Virage</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1-039||LPA||295||VIDE</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>JARDIN BOTANIQUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1-092||SOPIE||290||Pharmacie marina</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Pharmacie marina</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1-107||MARINA||290||Pharmacie marina</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CITE MARINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1-442||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>CITE COLOMBE 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1-124||ORANGE AKENDJE||290||Panneau Akandjé</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>VILLAGE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1-125||AGO RITA||290||Maquis Coup de Frein</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>CARREFOUR COUP FREIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1-125||AGO RITA||290||Pharmacie Saint Silvestre</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>A201||CITE DES CADRES||233||chez les Achi</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>CITE DES CADRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>A201||CITE DES CADRES||233||CSM Angre John Wesley</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>A321||||268||KFC</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BELLE VUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>A321||||268||Bibliothèque du lycée technique d'Abidjan</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>278||||270||VIDE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>R330 B||VOODOO||269||VIDE</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1-405||||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>CARREFOUR MIAMI BEACH NON LOIN FRANCK KESSIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1-370||||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>CARREFOUR MIAMI BEACH A DROITE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1-369||||298||Auchan</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>CARREFOUR BCEAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1-352||||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ABATTA 40 HECTARE DERRIERE CITE DON MELO 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1-237||||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ABTTA VILLAGE ESPACE KAFOLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1-323||||298||Maquis No Limit</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1-323||||298||Centre de santé communautaire d'Akouedo-Attie</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ABATTA AKOUEDO ATTIE ECOLE PRIMAIRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1-323||||298||Hôtel Nea 1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1-131||SCI LA FAMILLE||298||VIDE</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ABATTA DERRIERE ECOLE DES FAMILLES ETIMOE</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1-011||CENTRE DES ELEVEURS||295||VIDE</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>AGRICULTURE PROLONGEMENT EMPT VERS CITE DELACELLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1-106||FIGUIERS||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>FEH KESSEH FIGUIER 1 N/L PHARMACIE NISSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1-142||BELLE VUE||292||Cité Bellevue</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1-142||BELLE VUE||253||Cité Bellevue</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1-153||B.A.P||290||Anader</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ANADER PRES BROU AKA</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1-386||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>AKANDJE EXTENSION COTE GAUCHE AVANT PHARMACIE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1-388||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>AKANDJE APRES LA MOSQUEE GRANDE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1-383||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>AKANDJE JUSTE AVANT LE VILLAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1-346||||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>PARIS VILLAGE-MITTERAND PRES DE DOCTEUR PITTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1-155||LEWS HOLDIND||296||Pizza Eden</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1-155||LEWS HOLDIND||294||Morning Glory International School</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1-155||LEWS HOLDIND||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>LEWS HOLDING ENTREPRISE ( PRES HOTEL FREE WORLD )</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1-351||SIM BUSINESS LIMITED||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>AKANDJE PRES DU GROUPE SCOLAIRE LA POYANNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1-336||||290||Paroisse (chef Dago)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SANTE VILLAGE PRES DU TERRAIN ET DE LA PAROISSE ST MARCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1-138 B||||290||Hôtel Paris Village</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Hôtel Paris Village</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1-138 B||||290||Domicile DEK2</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1-270||REFLEXION||290||Maquis Chez Philippe</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ENVIRON HOTEL FREE WORLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1-266||||290||Paroisse (chef Dago)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SANTE VILLAGE NON PHARMACIE LES COLOMBES-EGLISE CATHOLIQUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1-252||OP IMM EBURNEENES||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>CITE EBURNEENE (SCIAM BTP)-ROUTE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1-245||SODIMEL||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>AKANDJE APRES PHARMACIE-MOSQUEE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1-075||AKENDJE||290||Panneau Akandjé</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>AKANDJE VILLAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1-172||AKENDJE 2||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>AKANDJE PERFORMER-UNIVERSITE POLYTECHNIQUE BINGERVILLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1-207||POHOU||290||Espace Nao</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ROUTE AKANDJE ESPACE NAMIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1-186||ETAMY-CI||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>AKANDJE PERFORMER B - CENTRE D EQUITATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1-022||AKOUAI SANTAI||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SANTE VILLAGE PRES ECOLE PRIMAIRE SANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1-175||CITE PERFORMER||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>AKANDJE PERFORMER B - PERFORMER A - PHARMACIE AKANDJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1-223||CITE COLOMBE 2||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ROUTE AKANDJE CITE COLOMBE 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1-173||||290||Pharmacie marina</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>PHARMACIE MARINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1-173||||290||Maquis Chez Philippe</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1-141||ADE MANSAH||290||Pharmacie marina</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CITE ALOBEE ADEMANSAH - FACE PHARMACIE MARINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1-208||PONDEUSE DE BRIQUE||294||Morning Glory International School</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1-208||PONDEUSE DE BRIQUE||296||Pizza Eden</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1-208||PONDEUSE DE BRIQUE||290||VIDE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>FABRIQUE DE BRIQUE - CARREFOUR HOTEL FREE WORLD</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>